<commit_message>
Track currency conversions separately from spend and income
</commit_message>
<xml_diff>
--- a/mock-data.xlsx
+++ b/mock-data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="72">
   <si>
     <t>Date</t>
   </si>
@@ -149,12 +149,18 @@
     <t>Special Expenses</t>
   </si>
   <si>
+    <t>Conversions</t>
+  </si>
+  <si>
     <t>Currencies</t>
   </si>
   <si>
     <t>School Fees</t>
   </si>
   <si>
+    <t>Conversion</t>
+  </si>
+  <si>
     <t>Clothes</t>
   </si>
   <si>
@@ -185,7 +191,7 @@
     <t>Electronics</t>
   </si>
   <si>
-    <t>Conversion</t>
+    <t>Investment Buy</t>
   </si>
   <si>
     <t>Loan</t>
@@ -194,9 +200,6 @@
     <t>Food General</t>
   </si>
   <si>
-    <t>Investment Buy</t>
-  </si>
-  <si>
     <t>Other Money in</t>
   </si>
   <si>
@@ -206,16 +209,16 @@
     <t>Investment Sell</t>
   </si>
   <si>
+    <t>Dividend</t>
+  </si>
+  <si>
     <t>Necessity</t>
   </si>
   <si>
-    <t>Dividend</t>
+    <t>Interest</t>
   </si>
   <si>
     <t>Medical</t>
-  </si>
-  <si>
-    <t>Interest</t>
   </si>
   <si>
     <t>Budgets</t>
@@ -3235,7 +3238,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -3246,7 +3249,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>42</v>
       </c>
@@ -3262,8 +3265,11 @@
       <c r="E2" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3271,33 +3277,36 @@
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -3305,27 +3314,27 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3333,32 +3342,29 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3366,28 +3372,25 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3395,10 +3398,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add per-currency symbols from the Constants sheet; migrate the interactive UI to Shoelace (dialogs, buttons, inputs)
</commit_message>
<xml_diff>
--- a/mock-data.xlsx
+++ b/mock-data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="74">
   <si>
     <t>Date</t>
   </si>
@@ -155,10 +155,16 @@
     <t>Currencies</t>
   </si>
   <si>
+    <t>Symbols</t>
+  </si>
+  <si>
     <t>School Fees</t>
   </si>
   <si>
     <t>Conversion</t>
+  </si>
+  <si>
+    <t>$</t>
   </si>
   <si>
     <t>Clothes</t>
@@ -3238,7 +3244,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -3249,7 +3255,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>42</v>
       </c>
@@ -3268,8 +3274,11 @@
       <c r="F2" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3277,36 +3286,42 @@
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -3314,27 +3329,30 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
       </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -3342,29 +3360,29 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -3372,25 +3390,25 @@
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3398,10 +3416,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>